<commit_message>
Clarify price adjustment in NVS source note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/NVS.xlsx
+++ b/models/NVS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zjult\ClaudeCode\biopharma-financial-models\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5CD223-F8E1-4887-A1D1-8EF5808403B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E16196C-69A0-4526-9F7D-0A0735EBFF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44055" yWindow="1530" windowWidth="19995" windowHeight="13635" xr2:uid="{F0652295-93CC-4638-BE61-190A5FE627D9}"/>
   </bookViews>
@@ -47,9 +47,6 @@
     <t>Novartis AG (NVS) - Daily Stock Price, Last 5 Years</t>
   </si>
   <si>
-    <t>Source: Nasdaq historical quotes (nasdaq.com/market-activity/stocks/nvs), retrieved 2026-10-05. Prices in USD per ADS; not split/dividend adjusted beyond Nasdaq's own presentation.</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
   </si>
   <si>
     <t>Volume (shares)</t>
+  </si>
+  <si>
+    <t>Source: Nasdaq historical quotes (nasdaq.com/market-activity/stocks/nvs), retrieved 2026-10-05. USD per ADS. Prices before 2023-10-03 are as adjusted by Nasdaq (4-decimal values), consistent with the Oct 2023 Sandoz spin-off.</t>
   </si>
 </sst>
 </file>
@@ -503,27 +503,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>